<commit_message>
add non_network_walk to scoring
</commit_message>
<xml_diff>
--- a/test/input/scenarios/mobi50test/scoringParametersIT.xlsx
+++ b/test/input/scenarios/mobi50test/scoringParametersIT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11027"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28827"/>
   <workbookPr date1904="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/annevaleriepreto/Documents/EPFL/matsim-sbb/test/input/scenarios/mobi50test/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\devsbb\code\matsim-sbb\test\input\scenarios\mobi50test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2BCDBFA-4C7D-6845-94DC-91F300C98923}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F23F66E-61AB-43A3-B71C-2D75BB4A02EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="140" yWindow="900" windowWidth="29080" windowHeight="18060" tabRatio="674" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="674" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScoringParams" sheetId="25" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="72">
   <si>
     <t>adaptation time</t>
   </si>
@@ -250,6 +250,9 @@
   </si>
   <si>
     <t>other</t>
+  </si>
+  <si>
+    <t>non_network_walk</t>
   </si>
 </sst>
 </file>
@@ -935,7 +938,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="6">
     <dxf>
@@ -1352,31 +1355,31 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:X22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <dimension ref="A1:Y22"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="30.33203125" customWidth="1"/>
-    <col min="2" max="2" width="19.5" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="1" max="1" width="30.28515625" customWidth="1"/>
+    <col min="2" max="2" width="19.42578125" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" customWidth="1"/>
     <col min="4" max="6" width="10" customWidth="1"/>
-    <col min="7" max="11" width="11.33203125" customWidth="1"/>
-    <col min="12" max="12" width="12.1640625" customWidth="1"/>
-    <col min="13" max="16" width="12.5" customWidth="1"/>
-    <col min="17" max="17" width="10.33203125" customWidth="1"/>
-    <col min="18" max="18" width="10.1640625" customWidth="1"/>
-    <col min="19" max="19" width="5.5" style="2" customWidth="1"/>
-    <col min="20" max="20" width="33.6640625" customWidth="1"/>
-    <col min="23" max="23" width="24.5" style="1" customWidth="1"/>
-    <col min="24" max="24" width="8.5" style="1" customWidth="1"/>
-    <col min="26" max="28" width="7.83203125" customWidth="1"/>
-    <col min="29" max="29" width="7.33203125" customWidth="1"/>
-    <col min="30" max="30" width="7.83203125" customWidth="1"/>
-    <col min="31" max="31" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="32" max="34" width="7.83203125" customWidth="1"/>
-    <col min="35" max="35" width="28" bestFit="1" customWidth="1"/>
+    <col min="7" max="11" width="11.28515625" customWidth="1"/>
+    <col min="12" max="13" width="12.140625" customWidth="1"/>
+    <col min="14" max="17" width="12.42578125" customWidth="1"/>
+    <col min="18" max="18" width="10.28515625" customWidth="1"/>
+    <col min="19" max="19" width="10.140625" customWidth="1"/>
+    <col min="20" max="20" width="5.42578125" style="2" customWidth="1"/>
+    <col min="21" max="21" width="33.7109375" customWidth="1"/>
+    <col min="24" max="24" width="24.42578125" style="1" customWidth="1"/>
+    <col min="25" max="25" width="8.42578125" style="1" customWidth="1"/>
+    <col min="27" max="29" width="7.85546875" customWidth="1"/>
+    <col min="30" max="30" width="7.28515625" customWidth="1"/>
+    <col min="31" max="31" width="7.85546875" customWidth="1"/>
+    <col min="32" max="32" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="33" max="35" width="7.85546875" customWidth="1"/>
+    <col min="36" max="36" width="28" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="50.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:21" ht="50.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="59" t="s">
         <v>64</v>
       </c>
@@ -1399,9 +1402,10 @@
       <c r="P1" s="123"/>
       <c r="Q1" s="123"/>
       <c r="R1" s="123"/>
-      <c r="S1" s="5"/>
+      <c r="S1" s="123"/>
+      <c r="T1" s="5"/>
     </row>
-    <row r="2" spans="1:20" ht="36" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
         <v>31</v>
       </c>
@@ -1436,27 +1440,30 @@
       <c r="L2" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="M2" s="22" t="s">
+      <c r="M2" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="N2" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="N2" s="22" t="s">
+      <c r="O2" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="O2" s="22" t="s">
+      <c r="P2" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="P2" s="23" t="s">
+      <c r="Q2" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="Q2" s="10" t="s">
+      <c r="R2" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="R2" s="9" t="s">
+      <c r="S2" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="S2" s="11"/>
+      <c r="T2" s="11"/>
     </row>
-    <row r="3" spans="1:20" ht="50.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:21" ht="50.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="17"/>
       <c r="B3" s="107" t="s">
         <v>15</v>
@@ -1491,30 +1498,33 @@
       <c r="L3" s="115" t="s">
         <v>51</v>
       </c>
-      <c r="M3" s="116" t="s">
+      <c r="M3" s="115" t="s">
+        <v>51</v>
+      </c>
+      <c r="N3" s="116" t="s">
         <v>55</v>
       </c>
-      <c r="N3" s="116" t="s">
+      <c r="O3" s="116" t="s">
         <v>56</v>
       </c>
-      <c r="O3" s="116" t="s">
+      <c r="P3" s="116" t="s">
         <v>57</v>
       </c>
-      <c r="P3" s="108" t="s">
+      <c r="Q3" s="108" t="s">
         <v>62</v>
       </c>
-      <c r="Q3" s="115" t="s">
+      <c r="R3" s="115" t="s">
         <v>59</v>
       </c>
-      <c r="R3" s="108" t="s">
+      <c r="S3" s="108" t="s">
         <v>28</v>
       </c>
-      <c r="S3" s="11"/>
-      <c r="T3" s="18" t="s">
+      <c r="T3" s="11"/>
+      <c r="U3" s="18" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:20" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:21" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="14" t="s">
         <v>2</v>
       </c>
@@ -1549,30 +1559,33 @@
       <c r="L4" s="84">
         <v>0</v>
       </c>
-      <c r="M4" s="120">
+      <c r="M4" s="84">
+        <v>0</v>
+      </c>
+      <c r="N4" s="120">
         <v>-0.43</v>
       </c>
-      <c r="N4" s="85">
+      <c r="O4" s="85">
         <v>-0.26</v>
       </c>
-      <c r="O4" s="85">
+      <c r="P4" s="85">
         <v>-0.06</v>
       </c>
-      <c r="P4" s="86">
+      <c r="Q4" s="86">
         <v>-0.17</v>
       </c>
-      <c r="Q4" s="84">
+      <c r="R4" s="84">
         <v>0.02</v>
       </c>
-      <c r="R4" s="86">
+      <c r="S4" s="86">
         <v>-0.24</v>
       </c>
-      <c r="S4" s="12"/>
-      <c r="T4" s="19" t="s">
+      <c r="T4" s="12"/>
+      <c r="U4" s="19" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:20" s="3" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:21" s="3" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="14" t="s">
         <v>14</v>
       </c>
@@ -1607,7 +1620,7 @@
       <c r="L5" s="81">
         <v>0</v>
       </c>
-      <c r="M5" s="82">
+      <c r="M5" s="81">
         <v>0</v>
       </c>
       <c r="N5" s="82">
@@ -1616,21 +1629,24 @@
       <c r="O5" s="82">
         <v>0</v>
       </c>
-      <c r="P5" s="83">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="81">
-        <v>0</v>
-      </c>
-      <c r="R5" s="82">
-        <v>0</v>
-      </c>
-      <c r="S5" s="12"/>
-      <c r="T5" s="20" t="s">
+      <c r="P5" s="82">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="83">
+        <v>0</v>
+      </c>
+      <c r="R5" s="81">
+        <v>0</v>
+      </c>
+      <c r="S5" s="82">
+        <v>0</v>
+      </c>
+      <c r="T5" s="12"/>
+      <c r="U5" s="20" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:20" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:21" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
         <v>13</v>
       </c>
@@ -1665,30 +1681,33 @@
       <c r="L6" s="47">
         <v>-0.31</v>
       </c>
-      <c r="M6" s="48">
+      <c r="M6" s="47">
+        <v>-0.31</v>
+      </c>
+      <c r="N6" s="48">
         <v>-0.22</v>
       </c>
-      <c r="N6" s="48">
+      <c r="O6" s="48">
         <v>-0.09</v>
       </c>
-      <c r="O6" s="48">
+      <c r="P6" s="48">
         <v>-0.57999999999999996</v>
       </c>
-      <c r="P6" s="80">
+      <c r="Q6" s="80">
         <v>-3.25</v>
       </c>
-      <c r="Q6" s="47">
+      <c r="R6" s="47">
         <v>-0.05</v>
       </c>
-      <c r="R6" s="48">
+      <c r="S6" s="48">
         <v>-0.7</v>
       </c>
-      <c r="S6" s="13"/>
-      <c r="T6" s="63" t="s">
+      <c r="T6" s="13"/>
+      <c r="U6" s="63" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:20" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:21" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="14" t="s">
         <v>12</v>
       </c>
@@ -1723,7 +1742,7 @@
       <c r="L7" s="81">
         <v>0</v>
       </c>
-      <c r="M7" s="82">
+      <c r="M7" s="81">
         <v>0</v>
       </c>
       <c r="N7" s="82">
@@ -1732,21 +1751,24 @@
       <c r="O7" s="82">
         <v>0</v>
       </c>
-      <c r="P7" s="83">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="81">
-        <v>0</v>
-      </c>
-      <c r="R7" s="82">
-        <v>0</v>
-      </c>
-      <c r="S7" s="11"/>
-      <c r="T7" s="124" t="s">
+      <c r="P7" s="82">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="83">
+        <v>0</v>
+      </c>
+      <c r="R7" s="81">
+        <v>0</v>
+      </c>
+      <c r="S7" s="82">
+        <v>0</v>
+      </c>
+      <c r="T7" s="11"/>
+      <c r="U7" s="124" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:20" ht="0.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:21" ht="0.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="14"/>
       <c r="B8" s="111"/>
       <c r="C8" s="34"/>
@@ -1775,7 +1797,7 @@
       <c r="L8" s="37" t="s">
         <v>66</v>
       </c>
-      <c r="M8" s="34" t="s">
+      <c r="M8" s="37" t="s">
         <v>66</v>
       </c>
       <c r="N8" s="34" t="s">
@@ -1784,19 +1806,22 @@
       <c r="O8" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="P8" s="118" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q8" s="37" t="s">
-        <v>66</v>
-      </c>
-      <c r="R8" s="36" t="s">
-        <v>66</v>
-      </c>
-      <c r="S8" s="11"/>
-      <c r="T8" s="124"/>
+      <c r="P8" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q8" s="118" t="s">
+        <v>66</v>
+      </c>
+      <c r="R8" s="37" t="s">
+        <v>66</v>
+      </c>
+      <c r="S8" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="T8" s="11"/>
+      <c r="U8" s="124"/>
     </row>
-    <row r="9" spans="1:20" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:21" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="15" t="s">
         <v>11</v>
       </c>
@@ -1827,7 +1852,7 @@
       <c r="L9" s="90" t="s">
         <v>66</v>
       </c>
-      <c r="M9" s="88" t="s">
+      <c r="M9" s="90" t="s">
         <v>66</v>
       </c>
       <c r="N9" s="88" t="s">
@@ -1836,19 +1861,22 @@
       <c r="O9" s="88" t="s">
         <v>66</v>
       </c>
-      <c r="P9" s="91" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q9" s="90" t="s">
-        <v>66</v>
-      </c>
-      <c r="R9" s="88" t="s">
-        <v>66</v>
-      </c>
-      <c r="S9" s="12"/>
-      <c r="T9" s="125"/>
+      <c r="P9" s="88" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q9" s="91" t="s">
+        <v>66</v>
+      </c>
+      <c r="R9" s="90" t="s">
+        <v>66</v>
+      </c>
+      <c r="S9" s="88" t="s">
+        <v>66</v>
+      </c>
+      <c r="T9" s="12"/>
+      <c r="U9" s="125"/>
     </row>
-    <row r="10" spans="1:20" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:21" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="14" t="s">
         <v>10</v>
       </c>
@@ -1879,7 +1907,7 @@
       <c r="L10" s="92" t="s">
         <v>66</v>
       </c>
-      <c r="M10" s="93" t="s">
+      <c r="M10" s="92" t="s">
         <v>66</v>
       </c>
       <c r="N10" s="93" t="s">
@@ -1888,18 +1916,21 @@
       <c r="O10" s="93" t="s">
         <v>66</v>
       </c>
-      <c r="P10" s="94" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q10" s="92" t="s">
-        <v>66</v>
-      </c>
-      <c r="R10" s="93" t="s">
-        <v>66</v>
-      </c>
-      <c r="S10" s="12"/>
+      <c r="P10" s="93" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q10" s="94" t="s">
+        <v>66</v>
+      </c>
+      <c r="R10" s="92" t="s">
+        <v>66</v>
+      </c>
+      <c r="S10" s="93" t="s">
+        <v>66</v>
+      </c>
+      <c r="T10" s="12"/>
     </row>
-    <row r="11" spans="1:20" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:21" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="15" t="s">
         <v>9</v>
       </c>
@@ -1930,7 +1961,7 @@
       <c r="L11" s="90" t="s">
         <v>66</v>
       </c>
-      <c r="M11" s="88" t="s">
+      <c r="M11" s="90" t="s">
         <v>66</v>
       </c>
       <c r="N11" s="88" t="s">
@@ -1939,18 +1970,21 @@
       <c r="O11" s="88" t="s">
         <v>66</v>
       </c>
-      <c r="P11" s="91" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q11" s="90" t="s">
-        <v>66</v>
-      </c>
-      <c r="R11" s="88" t="s">
-        <v>66</v>
-      </c>
-      <c r="S11" s="12"/>
+      <c r="P11" s="88" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q11" s="91" t="s">
+        <v>66</v>
+      </c>
+      <c r="R11" s="90" t="s">
+        <v>66</v>
+      </c>
+      <c r="S11" s="88" t="s">
+        <v>66</v>
+      </c>
+      <c r="T11" s="12"/>
     </row>
-    <row r="12" spans="1:20" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:21" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="14" t="s">
         <v>8</v>
       </c>
@@ -1981,7 +2015,7 @@
       <c r="L12" s="92" t="s">
         <v>66</v>
       </c>
-      <c r="M12" s="93" t="s">
+      <c r="M12" s="92" t="s">
         <v>66</v>
       </c>
       <c r="N12" s="93" t="s">
@@ -1990,18 +2024,21 @@
       <c r="O12" s="93" t="s">
         <v>66</v>
       </c>
-      <c r="P12" s="94" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q12" s="92" t="s">
-        <v>66</v>
-      </c>
-      <c r="R12" s="93" t="s">
-        <v>66</v>
-      </c>
-      <c r="S12" s="12"/>
+      <c r="P12" s="93" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q12" s="94" t="s">
+        <v>66</v>
+      </c>
+      <c r="R12" s="92" t="s">
+        <v>66</v>
+      </c>
+      <c r="S12" s="93" t="s">
+        <v>66</v>
+      </c>
+      <c r="T12" s="12"/>
     </row>
-    <row r="13" spans="1:20" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:21" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="14" t="s">
         <v>7</v>
       </c>
@@ -2032,7 +2069,7 @@
       <c r="L13" s="92" t="s">
         <v>66</v>
       </c>
-      <c r="M13" s="93" t="s">
+      <c r="M13" s="92" t="s">
         <v>66</v>
       </c>
       <c r="N13" s="93" t="s">
@@ -2041,18 +2078,21 @@
       <c r="O13" s="93" t="s">
         <v>66</v>
       </c>
-      <c r="P13" s="94" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q13" s="92" t="s">
-        <v>66</v>
-      </c>
-      <c r="R13" s="93" t="s">
-        <v>66</v>
-      </c>
-      <c r="S13" s="12"/>
+      <c r="P13" s="93" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q13" s="94" t="s">
+        <v>66</v>
+      </c>
+      <c r="R13" s="92" t="s">
+        <v>66</v>
+      </c>
+      <c r="S13" s="93" t="s">
+        <v>66</v>
+      </c>
+      <c r="T13" s="12"/>
     </row>
-    <row r="14" spans="1:20" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:21" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="14" t="s">
         <v>6</v>
       </c>
@@ -2083,7 +2123,7 @@
       <c r="L14" s="92" t="s">
         <v>66</v>
       </c>
-      <c r="M14" s="93" t="s">
+      <c r="M14" s="92" t="s">
         <v>66</v>
       </c>
       <c r="N14" s="93" t="s">
@@ -2092,18 +2132,21 @@
       <c r="O14" s="93" t="s">
         <v>66</v>
       </c>
-      <c r="P14" s="94" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q14" s="92" t="s">
-        <v>66</v>
-      </c>
-      <c r="R14" s="93" t="s">
-        <v>66</v>
-      </c>
-      <c r="S14" s="12"/>
+      <c r="P14" s="93" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q14" s="94" t="s">
+        <v>66</v>
+      </c>
+      <c r="R14" s="92" t="s">
+        <v>66</v>
+      </c>
+      <c r="S14" s="93" t="s">
+        <v>66</v>
+      </c>
+      <c r="T14" s="12"/>
     </row>
-    <row r="15" spans="1:20" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:21" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="16" t="s">
         <v>4</v>
       </c>
@@ -2140,27 +2183,30 @@
       <c r="L15" s="95">
         <v>0</v>
       </c>
-      <c r="M15" s="96">
+      <c r="M15" s="95">
+        <v>0</v>
+      </c>
+      <c r="N15" s="96">
         <v>0.05</v>
       </c>
-      <c r="N15" s="96">
+      <c r="O15" s="96">
         <v>0.14000000000000001</v>
       </c>
-      <c r="O15" s="96">
+      <c r="P15" s="96">
         <v>0.09</v>
       </c>
-      <c r="P15" s="97">
+      <c r="Q15" s="97">
         <v>0.1</v>
       </c>
-      <c r="Q15" s="95">
+      <c r="R15" s="95">
         <v>0.16</v>
       </c>
-      <c r="R15" s="96">
+      <c r="S15" s="96">
         <v>0.01</v>
       </c>
-      <c r="S15" s="12"/>
+      <c r="T15" s="12"/>
     </row>
-    <row r="16" spans="1:20" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:21" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="15" t="s">
         <v>41</v>
       </c>
@@ -2191,7 +2237,7 @@
       <c r="L16" s="98" t="s">
         <v>66</v>
       </c>
-      <c r="M16" s="100" t="s">
+      <c r="M16" s="98" t="s">
         <v>66</v>
       </c>
       <c r="N16" s="100" t="s">
@@ -2200,18 +2246,21 @@
       <c r="O16" s="100" t="s">
         <v>66</v>
       </c>
-      <c r="P16" s="99" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q16" s="98" t="s">
-        <v>66</v>
-      </c>
-      <c r="R16" s="99" t="s">
-        <v>66</v>
-      </c>
-      <c r="S16" s="4"/>
+      <c r="P16" s="100" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q16" s="99" t="s">
+        <v>66</v>
+      </c>
+      <c r="R16" s="98" t="s">
+        <v>66</v>
+      </c>
+      <c r="S16" s="99" t="s">
+        <v>66</v>
+      </c>
+      <c r="T16" s="4"/>
     </row>
-    <row r="17" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:20" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="14" t="s">
         <v>47</v>
       </c>
@@ -2242,7 +2291,7 @@
       <c r="L17" s="101" t="s">
         <v>66</v>
       </c>
-      <c r="M17" s="103" t="s">
+      <c r="M17" s="101" t="s">
         <v>66</v>
       </c>
       <c r="N17" s="103" t="s">
@@ -2251,18 +2300,21 @@
       <c r="O17" s="103" t="s">
         <v>66</v>
       </c>
-      <c r="P17" s="102" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q17" s="101" t="s">
-        <v>66</v>
-      </c>
-      <c r="R17" s="102" t="s">
-        <v>66</v>
-      </c>
-      <c r="S17" s="4"/>
+      <c r="P17" s="103" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q17" s="102" t="s">
+        <v>66</v>
+      </c>
+      <c r="R17" s="101" t="s">
+        <v>66</v>
+      </c>
+      <c r="S17" s="102" t="s">
+        <v>66</v>
+      </c>
+      <c r="T17" s="4"/>
     </row>
-    <row r="18" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:20" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="14" t="s">
         <v>43</v>
       </c>
@@ -2293,7 +2345,7 @@
       <c r="L18" s="101" t="s">
         <v>66</v>
       </c>
-      <c r="M18" s="103" t="s">
+      <c r="M18" s="101" t="s">
         <v>66</v>
       </c>
       <c r="N18" s="103" t="s">
@@ -2302,18 +2354,21 @@
       <c r="O18" s="103" t="s">
         <v>66</v>
       </c>
-      <c r="P18" s="102" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q18" s="101" t="s">
-        <v>66</v>
-      </c>
-      <c r="R18" s="102" t="s">
-        <v>66</v>
-      </c>
-      <c r="S18" s="4"/>
+      <c r="P18" s="103" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q18" s="102" t="s">
+        <v>66</v>
+      </c>
+      <c r="R18" s="101" t="s">
+        <v>66</v>
+      </c>
+      <c r="S18" s="102" t="s">
+        <v>66</v>
+      </c>
+      <c r="T18" s="4"/>
     </row>
-    <row r="19" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:20" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="14" t="s">
         <v>48</v>
       </c>
@@ -2344,7 +2399,7 @@
       <c r="L19" s="101" t="s">
         <v>66</v>
       </c>
-      <c r="M19" s="103" t="s">
+      <c r="M19" s="101" t="s">
         <v>66</v>
       </c>
       <c r="N19" s="103" t="s">
@@ -2353,18 +2408,21 @@
       <c r="O19" s="103" t="s">
         <v>66</v>
       </c>
-      <c r="P19" s="102" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q19" s="101" t="s">
-        <v>66</v>
-      </c>
-      <c r="R19" s="102" t="s">
-        <v>66</v>
-      </c>
-      <c r="S19" s="4"/>
+      <c r="P19" s="103" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q19" s="102" t="s">
+        <v>66</v>
+      </c>
+      <c r="R19" s="101" t="s">
+        <v>66</v>
+      </c>
+      <c r="S19" s="102" t="s">
+        <v>66</v>
+      </c>
+      <c r="T19" s="4"/>
     </row>
-    <row r="20" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:20" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="62" t="s">
         <v>49</v>
       </c>
@@ -2395,7 +2453,7 @@
       <c r="L20" s="104" t="s">
         <v>66</v>
       </c>
-      <c r="M20" s="106" t="s">
+      <c r="M20" s="104" t="s">
         <v>66</v>
       </c>
       <c r="N20" s="106" t="s">
@@ -2404,18 +2462,21 @@
       <c r="O20" s="106" t="s">
         <v>66</v>
       </c>
-      <c r="P20" s="105" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q20" s="104" t="s">
-        <v>66</v>
-      </c>
-      <c r="R20" s="105" t="s">
-        <v>66</v>
-      </c>
-      <c r="S20" s="4"/>
+      <c r="P20" s="106" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q20" s="105" t="s">
+        <v>66</v>
+      </c>
+      <c r="R20" s="104" t="s">
+        <v>66</v>
+      </c>
+      <c r="S20" s="105" t="s">
+        <v>66</v>
+      </c>
+      <c r="T20" s="4"/>
     </row>
-    <row r="21" spans="1:19" ht="3" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:20" ht="3" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="6"/>
@@ -2432,17 +2493,18 @@
       <c r="N21" s="7"/>
       <c r="O21" s="7"/>
       <c r="P21" s="7"/>
-      <c r="Q21" s="6"/>
+      <c r="Q21" s="7"/>
       <c r="R21" s="6"/>
-      <c r="S21" s="4"/>
+      <c r="S21" s="6"/>
+      <c r="T21" s="4"/>
     </row>
-    <row r="22" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="S22" s="4"/>
+    <row r="22" spans="1:20" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="T22" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B1:R1"/>
-    <mergeCell ref="T7:T9"/>
+    <mergeCell ref="B1:S1"/>
+    <mergeCell ref="U7:U9"/>
   </mergeCells>
   <pageMargins left="0.31496062992125984" right="0.31496062992125984" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="8" scale="90" orientation="landscape" r:id="rId1"/>
@@ -2455,47 +2517,47 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Tabelle3"/>
-  <dimension ref="A1:AE10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <dimension ref="A1:AF10"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="30.5" customWidth="1"/>
-    <col min="2" max="2" width="29.5" customWidth="1"/>
-    <col min="3" max="3" width="11.1640625" customWidth="1"/>
-    <col min="4" max="5" width="9.6640625" customWidth="1"/>
-    <col min="6" max="6" width="10.1640625" customWidth="1"/>
-    <col min="7" max="12" width="9.6640625" customWidth="1"/>
-    <col min="13" max="16" width="12.5" customWidth="1"/>
-    <col min="17" max="17" width="10.5" customWidth="1"/>
-    <col min="18" max="18" width="9.6640625" customWidth="1"/>
-    <col min="19" max="19" width="8.5" customWidth="1"/>
-    <col min="20" max="20" width="13.1640625" customWidth="1"/>
-    <col min="21" max="21" width="10.1640625" customWidth="1"/>
-    <col min="23" max="25" width="10.1640625" customWidth="1"/>
-    <col min="26" max="29" width="12.5" customWidth="1"/>
-    <col min="30" max="31" width="10.1640625" customWidth="1"/>
+    <col min="1" max="1" width="30.42578125" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" customWidth="1"/>
+    <col min="3" max="3" width="11.140625" customWidth="1"/>
+    <col min="4" max="5" width="9.7109375" customWidth="1"/>
+    <col min="6" max="6" width="10.140625" customWidth="1"/>
+    <col min="7" max="13" width="9.7109375" customWidth="1"/>
+    <col min="14" max="17" width="12.42578125" customWidth="1"/>
+    <col min="18" max="18" width="10.42578125" customWidth="1"/>
+    <col min="19" max="19" width="9.7109375" customWidth="1"/>
+    <col min="20" max="20" width="8.42578125" customWidth="1"/>
+    <col min="21" max="21" width="13.140625" customWidth="1"/>
+    <col min="22" max="22" width="10.140625" customWidth="1"/>
+    <col min="24" max="26" width="10.140625" customWidth="1"/>
+    <col min="27" max="30" width="12.42578125" customWidth="1"/>
+    <col min="31" max="32" width="10.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="50.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:32" ht="50.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="61" t="str">
         <f>ScoringParams!A1</f>
         <v>mobi31test</v>
       </c>
-      <c r="T1" s="5"/>
-      <c r="AB1" s="1"/>
+      <c r="U1" s="5"/>
       <c r="AC1" s="1"/>
+      <c r="AD1" s="1"/>
     </row>
-    <row r="2" spans="1:31" s="25" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:32" s="25" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="60" t="s">
         <v>35</v>
       </c>
       <c r="C2" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="T2" s="25" t="s">
+      <c r="U2" s="25" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:31" ht="34.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:32" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="26" t="s">
         <v>36</v>
       </c>
@@ -2531,73 +2593,76 @@
         <v>26</v>
       </c>
       <c r="M3" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="N3" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="N3" s="22" t="s">
+      <c r="O3" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="O3" s="22" t="s">
+      <c r="P3" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="P3" s="22" t="s">
+      <c r="Q3" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="Q3" s="22" t="s">
+      <c r="R3" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="R3" s="23" t="s">
+      <c r="S3" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="T3" s="21" t="str">
+      <c r="U3" s="21" t="str">
         <f>C3</f>
         <v>global</v>
       </c>
-      <c r="U3" s="21" t="str">
+      <c r="V3" s="21" t="str">
         <f>D3</f>
         <v>car</v>
       </c>
-      <c r="V3" s="22" t="str">
+      <c r="W3" s="22" t="str">
         <f>E3</f>
         <v>ride</v>
       </c>
-      <c r="W3" s="22" t="str">
+      <c r="X3" s="22" t="str">
         <f>F3</f>
         <v>avtaxi</v>
       </c>
-      <c r="X3" s="22" t="str">
+      <c r="Y3" s="22" t="str">
         <f>G3</f>
         <v>pt</v>
       </c>
-      <c r="Y3" s="22" t="str">
-        <f t="shared" ref="Y3:AE3" si="0">L3</f>
-        <v>walk</v>
-      </c>
       <c r="Z3" s="22" t="str">
+        <f t="shared" ref="Z3:AF3" si="0">M3</f>
+        <v>non_network_walk</v>
+      </c>
+      <c r="AA3" s="22" t="str">
         <f t="shared" si="0"/>
         <v>car_feeder</v>
       </c>
-      <c r="AA3" s="22" t="str">
+      <c r="AB3" s="22" t="str">
         <f t="shared" si="0"/>
         <v>ride_feeder</v>
       </c>
-      <c r="AB3" s="22" t="str">
+      <c r="AC3" s="22" t="str">
         <f t="shared" si="0"/>
         <v>bike_feeder</v>
       </c>
-      <c r="AC3" s="22" t="str">
+      <c r="AD3" s="22" t="str">
         <f t="shared" si="0"/>
         <v>av_feeder</v>
       </c>
-      <c r="AD3" s="22" t="str">
+      <c r="AE3" s="22" t="str">
         <f t="shared" si="0"/>
         <v>walk_main</v>
       </c>
-      <c r="AE3" s="23" t="str">
+      <c r="AF3" s="23" t="str">
         <f t="shared" si="0"/>
         <v>bike</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A4" s="38" t="s">
         <v>37</v>
       </c>
@@ -2647,56 +2712,59 @@
       <c r="Q4" s="28">
         <v>0</v>
       </c>
-      <c r="R4" s="31">
-        <v>0</v>
-      </c>
-      <c r="T4" s="65"/>
-      <c r="U4" s="57">
+      <c r="R4" s="28">
+        <v>0</v>
+      </c>
+      <c r="S4" s="31">
+        <v>0</v>
+      </c>
+      <c r="U4" s="65"/>
+      <c r="V4" s="57">
         <f>D4+ScoringParams!D4</f>
         <v>-7.0000000000000007E-2</v>
       </c>
-      <c r="V4" s="58">
+      <c r="W4" s="58">
         <f>E4+ScoringParams!E4</f>
         <v>-0.7</v>
       </c>
-      <c r="W4" s="43">
+      <c r="X4" s="43">
         <f>F4+ScoringParams!F4</f>
         <v>0</v>
       </c>
-      <c r="X4" s="58">
+      <c r="Y4" s="58">
         <f>G4+ScoringParams!G4</f>
         <v>-0.02</v>
       </c>
-      <c r="Y4" s="58">
-        <f>L4+ScoringParams!L4</f>
-        <v>0</v>
-      </c>
       <c r="Z4" s="58">
-        <f>M4+ScoringParams!M4</f>
-        <v>-0.43</v>
+        <f>M4+ScoringParams!L4</f>
+        <v>0</v>
       </c>
       <c r="AA4" s="58">
         <f>N4+ScoringParams!N4</f>
+        <v>-0.43</v>
+      </c>
+      <c r="AB4" s="58">
+        <f>O4+ScoringParams!O4</f>
         <v>-0.26</v>
-      </c>
-      <c r="AB4" s="43">
-        <f>O4+ScoringParams!O4</f>
-        <v>-0.06</v>
       </c>
       <c r="AC4" s="43">
         <f>P4+ScoringParams!P4</f>
-        <v>-0.17</v>
+        <v>-0.06</v>
       </c>
       <c r="AD4" s="43">
         <f>Q4+ScoringParams!Q4</f>
+        <v>-0.17</v>
+      </c>
+      <c r="AE4" s="43">
+        <f>R4+ScoringParams!R4</f>
         <v>0.02</v>
       </c>
-      <c r="AE4" s="44">
-        <f>R4+ScoringParams!R4</f>
+      <c r="AF4" s="44">
+        <f>S4+ScoringParams!S4</f>
         <v>-0.24</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A5" s="39" t="s">
         <v>37</v>
       </c>
@@ -2731,7 +2799,7 @@
       <c r="L5" s="28">
         <v>0</v>
       </c>
-      <c r="M5" s="50">
+      <c r="M5" s="28">
         <v>0</v>
       </c>
       <c r="N5" s="50">
@@ -2743,42 +2811,41 @@
       <c r="P5" s="50">
         <v>0</v>
       </c>
-      <c r="Q5" s="28">
-        <v>0</v>
-      </c>
-      <c r="R5" s="31">
-        <v>0</v>
-      </c>
-      <c r="T5" s="69"/>
-      <c r="U5" s="35">
+      <c r="Q5" s="50">
+        <v>0</v>
+      </c>
+      <c r="R5" s="28">
+        <v>0</v>
+      </c>
+      <c r="S5" s="31">
+        <v>0</v>
+      </c>
+      <c r="U5" s="69"/>
+      <c r="V5" s="35">
         <f>D5+ScoringParams!D5</f>
         <v>-1.2E-5</v>
       </c>
-      <c r="V5" s="54">
+      <c r="W5" s="54">
         <f>E5+ScoringParams!E5</f>
         <v>-3.3000000000000002E-6</v>
       </c>
-      <c r="W5" s="45">
+      <c r="X5" s="45">
         <f>F5+ScoringParams!F5</f>
         <v>0</v>
       </c>
-      <c r="X5" s="54">
+      <c r="Y5" s="54">
         <f>G5+ScoringParams!G5</f>
         <v>1.5E-5</v>
       </c>
-      <c r="Y5" s="54">
-        <f>L5+ScoringParams!L5</f>
-        <v>0</v>
-      </c>
       <c r="Z5" s="54">
-        <f>M5+ScoringParams!M5</f>
+        <f>M5+ScoringParams!L5</f>
         <v>0</v>
       </c>
       <c r="AA5" s="54">
         <f>N5+ScoringParams!N5</f>
         <v>0</v>
       </c>
-      <c r="AB5" s="45">
+      <c r="AB5" s="54">
         <f>O5+ScoringParams!O5</f>
         <v>0</v>
       </c>
@@ -2790,12 +2857,16 @@
         <f>Q5+ScoringParams!Q5</f>
         <v>0</v>
       </c>
-      <c r="AE5" s="46">
+      <c r="AE5" s="45">
         <f>R5+ScoringParams!R5</f>
         <v>0</v>
       </c>
+      <c r="AF5" s="46">
+        <f>S5+ScoringParams!S5</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A6" s="39" t="s">
         <v>37</v>
       </c>
@@ -2845,56 +2916,59 @@
       <c r="Q6" s="28">
         <v>0</v>
       </c>
-      <c r="R6" s="31">
-        <v>0</v>
-      </c>
-      <c r="T6" s="69"/>
-      <c r="U6" s="37">
+      <c r="R6" s="28">
+        <v>0</v>
+      </c>
+      <c r="S6" s="31">
+        <v>0</v>
+      </c>
+      <c r="U6" s="69"/>
+      <c r="V6" s="37">
         <f>D6+ScoringParams!D6</f>
         <v>-0.44</v>
       </c>
-      <c r="V6" s="36">
+      <c r="W6" s="36">
         <f>E6+ScoringParams!E6</f>
         <v>-0.79</v>
       </c>
-      <c r="W6" s="45">
+      <c r="X6" s="45">
         <f>F6+ScoringParams!F6</f>
         <v>-0.17</v>
       </c>
-      <c r="X6" s="36">
+      <c r="Y6" s="36">
         <f>G6+ScoringParams!G6</f>
         <v>-7.0000000000000007E-2</v>
       </c>
-      <c r="Y6" s="36">
-        <f>L6+ScoringParams!L6</f>
+      <c r="Z6" s="36">
+        <f>M6+ScoringParams!L6</f>
         <v>-0.31</v>
-      </c>
-      <c r="Z6" s="36">
-        <f>M6+ScoringParams!M6</f>
-        <v>-0.22</v>
       </c>
       <c r="AA6" s="36">
         <f>N6+ScoringParams!N6</f>
+        <v>-0.22</v>
+      </c>
+      <c r="AB6" s="36">
+        <f>O6+ScoringParams!O6</f>
         <v>-0.09</v>
-      </c>
-      <c r="AB6" s="45">
-        <f>O6+ScoringParams!O6</f>
-        <v>-0.57999999999999996</v>
       </c>
       <c r="AC6" s="45">
         <f>P6+ScoringParams!P6</f>
-        <v>-3.25</v>
+        <v>-0.57999999999999996</v>
       </c>
       <c r="AD6" s="45">
         <f>Q6+ScoringParams!Q6</f>
+        <v>-3.25</v>
+      </c>
+      <c r="AE6" s="45">
+        <f>R6+ScoringParams!R6</f>
         <v>-0.05</v>
       </c>
-      <c r="AE6" s="46">
-        <f>R6+ScoringParams!R6</f>
+      <c r="AF6" s="46">
+        <f>S6+ScoringParams!S6</f>
         <v>-0.7</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A7" s="39" t="s">
         <v>37</v>
       </c>
@@ -2930,57 +3004,56 @@
         <v>0</v>
       </c>
       <c r="M7" s="29">
+        <v>0</v>
+      </c>
+      <c r="N7" s="29">
         <f>D7</f>
         <v>-2.1800000000000001E-4</v>
       </c>
-      <c r="N7" s="29">
+      <c r="O7" s="29">
         <f>E7</f>
         <v>-2.1800000000000001E-4</v>
       </c>
-      <c r="O7" s="29">
-        <v>0</v>
-      </c>
       <c r="P7" s="29">
         <v>0</v>
       </c>
       <c r="Q7" s="29">
         <v>0</v>
       </c>
-      <c r="R7" s="33">
-        <v>0</v>
-      </c>
-      <c r="T7" s="66"/>
-      <c r="U7" s="55">
+      <c r="R7" s="29">
+        <v>0</v>
+      </c>
+      <c r="S7" s="33">
+        <v>0</v>
+      </c>
+      <c r="U7" s="66"/>
+      <c r="V7" s="55">
         <f>D7+ScoringParams!D7</f>
         <v>-2.1800000000000001E-4</v>
       </c>
-      <c r="V7" s="56">
+      <c r="W7" s="56">
         <f>E7+ScoringParams!E7</f>
         <v>-2.1800000000000001E-4</v>
       </c>
-      <c r="W7" s="41">
+      <c r="X7" s="41">
         <f>F7+ScoringParams!F7</f>
         <v>0</v>
       </c>
-      <c r="X7" s="56">
+      <c r="Y7" s="56">
         <f>G7+ScoringParams!G7</f>
         <v>-3.4200000000000002E-4</v>
       </c>
-      <c r="Y7" s="56">
-        <f>L7+ScoringParams!L7</f>
-        <v>0</v>
-      </c>
       <c r="Z7" s="56">
-        <f>M7+ScoringParams!M7</f>
-        <v>-2.1800000000000001E-4</v>
+        <f>M7+ScoringParams!L7</f>
+        <v>0</v>
       </c>
       <c r="AA7" s="56">
         <f>N7+ScoringParams!N7</f>
         <v>-2.1800000000000001E-4</v>
       </c>
-      <c r="AB7" s="41">
+      <c r="AB7" s="56">
         <f>O7+ScoringParams!O7</f>
-        <v>0</v>
+        <v>-2.1800000000000001E-4</v>
       </c>
       <c r="AC7" s="41">
         <f>P7+ScoringParams!P7</f>
@@ -2990,12 +3063,16 @@
         <f>Q7+ScoringParams!Q7</f>
         <v>0</v>
       </c>
-      <c r="AE7" s="42">
+      <c r="AE7" s="41">
         <f>R7+ScoringParams!R7</f>
         <v>0</v>
       </c>
+      <c r="AF7" s="42">
+        <f>S7+ScoringParams!S7</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A8" s="38" t="s">
         <v>37</v>
       </c>
@@ -3005,12 +3082,12 @@
       <c r="C8" s="67">
         <v>0</v>
       </c>
-      <c r="T8" s="75">
+      <c r="U8" s="75">
         <f>C8+ScoringParams!C16</f>
         <v>-0.1</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A9" s="39" t="s">
         <v>37</v>
       </c>
@@ -3020,12 +3097,12 @@
       <c r="C9" s="70">
         <v>0</v>
       </c>
-      <c r="T9" s="76">
+      <c r="U9" s="76">
         <f>C9+ScoringParams!C17</f>
         <v>0.04</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A10" s="40" t="s">
         <v>37</v>
       </c>
@@ -3035,7 +3112,7 @@
       <c r="C10" s="68">
         <v>0</v>
       </c>
-      <c r="T10" s="77">
+      <c r="U10" s="77">
         <f>C10+ScoringParams!C18</f>
         <v>-0.16</v>
       </c>
@@ -3049,7 +3126,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D4:R7">
+  <conditionalFormatting sqref="D4:S7">
     <cfRule type="cellIs" dxfId="3" priority="5" operator="equal">
       <formula>0</formula>
     </cfRule>
@@ -3057,13 +3134,13 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T8:T10">
+  <conditionalFormatting sqref="U8:U10">
     <cfRule type="cellIs" dxfId="1" priority="14" operator="between">
       <formula>0</formula>
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U4:AE7">
+  <conditionalFormatting sqref="V4:AF7">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="between">
       <formula>0</formula>
       <formula>0</formula>

</xml_diff>